<commit_message>
make migrate & model
</commit_message>
<xml_diff>
--- a/scripts/output/merged_data_6089491.xlsx
+++ b/scripts/output/merged_data_6089491.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,25 +462,30 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Profile Photo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Bidang Minat</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>SINTA Score Overall</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>SINTA Score 3Yr</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Affil Score</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Affil Score 3Yr</t>
         </is>
@@ -505,17 +510,22 @@
       <c r="D2" t="n">
         <v>6089491</v>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="n">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://scholar.googleusercontent.com/citations?view_op=view_photo&amp;user=vRI8v3cAAAAJ&amp;citpid=1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
         <v>715</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>318</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>110</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>65</v>
       </c>
     </row>
@@ -1009,22 +1019,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Peran Ahli Patologi Klinis Dalam Memerangi Perdagangan Ilegal Obat Resep Terbatas Di Kabupaten Sleman, Daerah Istimewa Yogyakarta</t>
+          <t>Penegakan Hukum Tindak Pidana Perjudian Melalui Transaksi Informasi dan Elektronik: Studi Putusan Nomor 7104/K/Pid. Sus/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Peran Ahli Patologi Klinis Dalam Memerangi Perdagangan Ilegal Obat Resep Terbatas Di Kabupaten Sleman, Daerah Istimewa Yogyakarta'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Penegakan Hukum Tindak Pidana Perjudian Melalui Transaksi Informasi dan Elektronik: Studi Putusan Nomor 7104/K/Pid. Sus/2025'</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AS Sanggacita, H Irhamdessetya, AC Irawati</t>
+          <t>SO Devi, AC Irawati</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 283-290, 2026</t>
+          <t>Al-Zayn: Jurnal Ilmu Sosial &amp; Hukum 4 (1), 5574-5580, 2026</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -1071,22 +1081,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Keadilan Restoratif: Model Perlindungan Hukum Oleh Aparat Penegak Hukum (Polisi) Dalam Menangani Anak-Anak Yang Terlibat Dalam Perundungan</t>
+          <t>Optimasi Pemulihan Hak Korban Dalam Kasus Perundungan: Analisis Implementasi Pasal 9 Ayat (1a) Undang-Undang Perlindungan Anak</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Keadilan Restoratif: Model Perlindungan Hukum Oleh Aparat Penegak Hukum (Polisi) Dalam Menangani Anak-Anak Yang Terlibat Dalam Perundungan'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Optimasi Pemulihan Hak Korban Dalam Kasus Perundungan: Analisis Implementasi Pasal 9 Ayat (1a) Undang-Undang Perlindungan Anak'</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>W Winarti, AC Irawati</t>
+          <t>PM Sipahutar, AC Irawati</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 105-114, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 77-86, 2026</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -1102,22 +1112,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Penegakan Hukum Tindak Pidana Perjudian Melalui Transaksi Informasi dan Elektronik: Studi Putusan Nomor 7104/K/Pid. Sus/2025</t>
+          <t>Implementasi Penegakan Peraturan Daerah (Perda) Ketentraman Masyarakat Dan Perlindungan Masyarakat Di Kabupaten Semarang</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Penegakan Hukum Tindak Pidana Perjudian Melalui Transaksi Informasi dan Elektronik: Studi Putusan Nomor 7104/K/Pid. Sus/2025'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Implementasi Penegakan Peraturan Daerah (Perda) Ketentraman Masyarakat Dan Perlindungan Masyarakat Di Kabupaten Semarang'</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SO Devi, AC Irawati</t>
+          <t>AK Devi, I Yuliawan, AC Irawati</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Al-Zayn: Jurnal Ilmu Sosial &amp; Hukum 4 (1), 5574-5580, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 234-241, 2026</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1133,22 +1143,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Penegakan Hukum Tindakan Kriminal Yang Dilakukan Dalam Perjudian Online Oleh Anak-Anak (Studi Kasus Di Kepolisian Metropolitan Semarang)</t>
+          <t>Pejabat Desa Indonesia Dalam Upaya Mencari Kejelasan Hukum Mengenai Status Pekerjaan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Penegakan Hukum Tindakan Kriminal Yang Dilakukan Dalam Perjudian Online Oleh Anak-Anak (Studi Kasus Di Kepolisian Metropolitan Semarang)'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Pejabat Desa Indonesia Dalam Upaya Mencari Kejelasan Hukum Mengenai Status Pekerjaan'</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>AC Irawati</t>
+          <t>T Triyono, AC Irawati</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 181-190, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 124-131, 2026</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -1195,22 +1205,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Implementasi Ketentuan Batas Usia Dewasa dalam Pelayanan Hukum dan Administrasi Kependudukan pada Pemerintah Desa Mejagong, Kecamatan Randudongkal, Kabupaten Pemalang.</t>
+          <t>Penipuan Berbasis Online Di Kota Semarang: Analisis Yuridis-Normatif Dalam Perspektif Hukum Pidana</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Implementasi Ketentuan Batas Usia Dewasa dalam Pelayanan Hukum dan Administrasi Kependudukan pada Pemerintah Desa Mejagong, Kecamatan Randudongkal, Kabupaten Pemalang.'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Penipuan Berbasis Online Di Kota Semarang: Analisis Yuridis-Normatif Dalam Perspektif Hukum Pidana'</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>S Sonhaji, AC Irawati</t>
+          <t>TD Satria, H Irhamdesstya, AC Irawati</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 242-250, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 251-259, 2026</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -1226,29 +1236,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Urgensi Kesadaran Digital dalam Mewujudkan Ruang Aman melalui Literasi Digital dan Penerapan Proporsional Undang-Undang ITE</t>
+          <t>Pendekatan Hukum Terhadap Pembangunan Teknologi Informasi Dan Perlindungan Data Pribadi</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Urgensi Kesadaran Digital dalam Mewujudkan Ruang Aman melalui Literasi Digital dan Penerapan Proporsional Undang-Undang ITE'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Pendekatan Hukum Terhadap Pembangunan Teknologi Informasi Dan Perlindungan Data Pribadi'</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>F Budiarti, H Irhamdesetya, AC Irawati</t>
+          <t>G Aulia, AC Irawati</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 142-151, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 115-123, 2026</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>2026</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1257,22 +1267,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Penjatuhan Pidana Dalam Tindak Pidana Kekerasan Dalam Rumah Tangga Mewujudkan Kepastian Hukum: Studi Putusan Nomor 121/Pid. Sus/2025/PN Pti</t>
+          <t>Penegakan Hukum Tindakan Kriminal Yang Dilakukan Dalam Perjudian Online Oleh Anak-Anak (Studi Kasus Di Kepolisian Metropolitan Semarang)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Penjatuhan Pidana Dalam Tindak Pidana Kekerasan Dalam Rumah Tangga Mewujudkan Kepastian Hukum: Studi Putusan Nomor 121/Pid. Sus/2025/PN Pti'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Penegakan Hukum Tindakan Kriminal Yang Dilakukan Dalam Perjudian Online Oleh Anak-Anak (Studi Kasus Di Kepolisian Metropolitan Semarang)'</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>QM Ulfa, AC Irawati</t>
+          <t>AC Irawati</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Al-Zayn: Jurnal Ilmu Sosial &amp; Hukum 4 (1), 5827-5832, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 181-190, 2026</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -1288,22 +1298,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Model Penegakan Hukum Pada Tindak Pidana Pencurian Anak Melalui Diversi: Studi Putusan Nomor 7/Pid. Sus-Anak/2025/PN Unr</t>
+          <t>Peran Ahli Patologi Klinis Dalam Memerangi Perdagangan Ilegal Obat Resep Terbatas Di Kabupaten Sleman, Daerah Istimewa Yogyakarta</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Model Penegakan Hukum Pada Tindak Pidana Pencurian Anak Melalui Diversi: Studi Putusan Nomor 7/Pid. Sus-Anak/2025/PN Unr'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Peran Ahli Patologi Klinis Dalam Memerangi Perdagangan Ilegal Obat Resep Terbatas Di Kabupaten Sleman, Daerah Istimewa Yogyakarta'</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SO Devi, AC Irawati</t>
+          <t>AS Sanggacita, H Irhamdessetya, AC Irawati</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Al-Zayn: Jurnal Ilmu Sosial &amp; Hukum 4 (1), 5566-5573, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 283-290, 2026</t>
         </is>
       </c>
       <c r="F11" t="n">

</xml_diff>

<commit_message>
kontrol panel dosen s2
</commit_message>
<xml_diff>
--- a/scripts/output/merged_data_6089491.xlsx
+++ b/scripts/output/merged_data_6089491.xlsx
@@ -1019,22 +1019,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Penjatuhan Pidana Dalam Tindak Pidana Kekerasan Dalam Rumah Tangga Mewujudkan Kepastian Hukum: Studi Putusan Nomor 121/Pid. Sus/2025/PN Pti</t>
+          <t>Penegakan Hukum Tindak Pidana Perjudian Melalui Transaksi Informasi dan Elektronik: Studi Putusan Nomor 7104/K/Pid. Sus/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Penjatuhan Pidana Dalam Tindak Pidana Kekerasan Dalam Rumah Tangga Mewujudkan Kepastian Hukum: Studi Putusan Nomor 121/Pid. Sus/2025/PN Pti'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Penegakan Hukum Tindak Pidana Perjudian Melalui Transaksi Informasi dan Elektronik: Studi Putusan Nomor 7104/K/Pid. Sus/2025'</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>QM Ulfa, AC Irawati</t>
+          <t>SO Devi, AC Irawati</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Al-Zayn: Jurnal Ilmu Sosial &amp; Hukum 4 (1), 5827-5832, 2026</t>
+          <t>Al-Zayn: Jurnal Ilmu Sosial &amp; Hukum 4 (1), 5574-5580, 2026</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -1050,22 +1050,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Implementasi Penegakan Peraturan Daerah (Perda) Ketentraman Masyarakat Dan Perlindungan Masyarakat Di Kabupaten Semarang</t>
+          <t>Penegakan Hukum Tindakan Kriminal Yang Dilakukan Dalam Perjudian Online Oleh Anak-Anak (Studi Kasus Di Kepolisian Metropolitan Semarang)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Implementasi Penegakan Peraturan Daerah (Perda) Ketentraman Masyarakat Dan Perlindungan Masyarakat Di Kabupaten Semarang'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Penegakan Hukum Tindakan Kriminal Yang Dilakukan Dalam Perjudian Online Oleh Anak-Anak (Studi Kasus Di Kepolisian Metropolitan Semarang)'</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AK Devi, I Yuliawan, AC Irawati</t>
+          <t>AC Irawati</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 234-241, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 181-190, 2026</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -1081,22 +1081,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Keadilan Restoratif: Model Perlindungan Hukum Oleh Aparat Penegak Hukum (Polisi) Dalam Menangani Anak-Anak Yang Terlibat Dalam Perundungan</t>
+          <t>Criminal Responsibility of Business Actors for The Distribution of Food Containing Dangerous Substances</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Keadilan Restoratif: Model Perlindungan Hukum Oleh Aparat Penegak Hukum (Polisi) Dalam Menangani Anak-Anak Yang Terlibat Dalam Perundungan'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Criminal Responsibility of Business Actors for The Distribution of Food Containing Dangerous Substances'</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>W Winarti, AC Irawati</t>
+          <t>W Waryadi, AC Irawati</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 105-114, 2026</t>
+          <t>UNTAG Law Review 9 (2), 82-92, 2026</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -1112,22 +1112,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dominasi Kepentingan Partai Politik Dalam Proses Legislasi Di Dpr: Sebuah Studi Hukum Konstitusi</t>
+          <t>Peran Ahli Patologi Klinis Dalam Memerangi Perdagangan Ilegal Obat Resep Terbatas Di Kabupaten Sleman, Daerah Istimewa Yogyakarta</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Dominasi Kepentingan Partai Politik Dalam Proses Legislasi Di Dpr: Sebuah Studi Hukum Konstitusi'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Peran Ahli Patologi Klinis Dalam Memerangi Perdagangan Ilegal Obat Resep Terbatas Di Kabupaten Sleman, Daerah Istimewa Yogyakarta'</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>S Sholehuddin, AC Irawati</t>
+          <t>AS Sanggacita, H Irhamdessetya, AC Irawati</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 291-299, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 283-290, 2026</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1143,22 +1143,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dominasi Kepentingan Partai Politik Dalam Proses Legislasi Di Dpr: Sebuah Studi Hukum Konstitusi</t>
+          <t>Penerapan Demokrasi Partisipatif Untuk Memperkuat Tata Kelola Desa Yang Baik</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Dominasi Kepentingan Partai Politik Dalam Proses Legislasi Di Dpr: Sebuah Studi Hukum Konstitusi'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Penerapan Demokrasi Partisipatif Untuk Memperkuat Tata Kelola Desa Yang Baik'</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>S Sholehuddin, AC Irawati</t>
+          <t>KA Saputra, M Lativ, AC Irawati</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 291-299, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 227-233, 2026</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -1174,22 +1174,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Penjatuhan Pidana Dalam Tindak Pidana Kekerasan Dalam Rumah Tangga Ditinjau Dari Asas Keadilan Retributif</t>
+          <t>Keadilan Restoratif: Model Perlindungan Hukum Oleh Aparat Penegak Hukum (Polisi) Dalam Menangani Anak-Anak Yang Terlibat Dalam Perundungan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Penjatuhan Pidana Dalam Tindak Pidana Kekerasan Dalam Rumah Tangga Ditinjau Dari Asas Keadilan Retributif'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Keadilan Restoratif: Model Perlindungan Hukum Oleh Aparat Penegak Hukum (Polisi) Dalam Menangani Anak-Anak Yang Terlibat Dalam Perundungan'</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>HN Hanifah, AC Irawati</t>
+          <t>W Winarti, AC Irawati</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Jurnal Pengabdian Masyarakat dan Riset Pendidikan 4 (3), 20402-20404, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 105-114, 2026</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -1205,29 +1205,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PERLINDUNGAN DATA PRIBADI SEBAGAI INSTRUMEN HUKUM DALAM MENANGGULANGI KEJAHATAN PERBANKAN</t>
+          <t>Model Penegakan Hukum Pada Tindak Pidana Pencurian Anak Melalui Diversi: Studi Putusan Nomor 7/Pid. Sus-Anak/2025/PN Unr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'PERLINDUNGAN DATA PRIBADI SEBAGAI INSTRUMEN HUKUM DALAM MENANGGULANGI KEJAHATAN PERBANKAN'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Model Penegakan Hukum Pada Tindak Pidana Pencurian Anak Melalui Diversi: Studi Putusan Nomor 7/Pid. Sus-Anak/2025/PN Unr'</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>N Sugiarto, I Yuliawan, AC Irawati</t>
+          <t>SO Devi, AC Irawati</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Pendas: Jurnal Ilmiah Pendidikan Dasar 11 (01), 260-275, 2026</t>
+          <t>Al-Zayn: Jurnal Ilmu Sosial &amp; Hukum 4 (1), 5566-5573, 2026</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>2026</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1236,22 +1236,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Penjatuhan Pidana Dalam Tindak Pidana Kekerasan Dalam Rumah Tangga Ditinjau Dari Asas Keadilan Retributif</t>
+          <t>Model Pencegahan Penarikan Kendaraan Leasing Melalui Komunikasi Proaktif Di Kota Semarang</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Penjatuhan Pidana Dalam Tindak Pidana Kekerasan Dalam Rumah Tangga Ditinjau Dari Asas Keadilan Retributif'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Model Pencegahan Penarikan Kendaraan Leasing Melalui Komunikasi Proaktif Di Kota Semarang'</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>HN Hanifah, AC Irawati</t>
+          <t>RD Saputra, H Irhamdesstya, AC Irawati</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Jurnal Pengabdian Masyarakat dan Riset Pendidikan 4 (3), 20402-20404, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 216-226, 2026</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1267,29 +1267,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Penerapan Undang-Undang Tentang Informasi Dan Transaksi Elektronik (Uu Ite) Dalam Kebebasan Berpendapat Dan Berekspresi</t>
+          <t>Implementasi E-Faktur Pajak Kendaraan Bermotor dalam Perspektif Hukum Administrasi Negara pada Polrestabes Semarang</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Penerapan Undang-Undang Tentang Informasi Dan Transaksi Elektronik (Uu Ite) Dalam Kebebasan Berpendapat Dan Berekspresi'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Implementasi E-Faktur Pajak Kendaraan Bermotor dalam Perspektif Hukum Administrasi Negara pada Polrestabes Semarang'</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>H Sinaga, AC Irawati</t>
+          <t>A Wijayanto, AC Irawati</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 172-180, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 68-76, 2026</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>2026</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1298,22 +1298,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Implementasi E-Faktur Pajak Kendaraan Bermotor dalam Perspektif Hukum Administrasi Negara pada Polrestabes Semarang</t>
+          <t>Implementasi Ketentuan Batas Usia Dewasa dalam Pelayanan Hukum dan Administrasi Kependudukan pada Pemerintah Desa Mejagong, Kecamatan Randudongkal, Kabupaten Pemalang.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Implementasi E-Faktur Pajak Kendaraan Bermotor dalam Perspektif Hukum Administrasi Negara pada Polrestabes Semarang'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Implementasi Ketentuan Batas Usia Dewasa dalam Pelayanan Hukum dan Administrasi Kependudukan pada Pemerintah Desa Mejagong, Kecamatan Randudongkal, Kabupaten Pemalang.'</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>A Wijayanto, AC Irawati</t>
+          <t>S Sonhaji, AC Irawati</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 68-76, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 242-250, 2026</t>
         </is>
       </c>
       <c r="F11" t="n">

</xml_diff>

<commit_message>
akademik header tidak statis
</commit_message>
<xml_diff>
--- a/scripts/output/merged_data_6089491.xlsx
+++ b/scripts/output/merged_data_6089491.xlsx
@@ -1019,22 +1019,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Penegakan Hukum Tindak Pidana Perjudian Melalui Transaksi Informasi dan Elektronik: Studi Putusan Nomor 7104/K/Pid. Sus/2025</t>
+          <t>Peran Ahli Patologi Klinis Dalam Memerangi Perdagangan Ilegal Obat Resep Terbatas Di Kabupaten Sleman, Daerah Istimewa Yogyakarta</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Penegakan Hukum Tindak Pidana Perjudian Melalui Transaksi Informasi dan Elektronik: Studi Putusan Nomor 7104/K/Pid. Sus/2025'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Peran Ahli Patologi Klinis Dalam Memerangi Perdagangan Ilegal Obat Resep Terbatas Di Kabupaten Sleman, Daerah Istimewa Yogyakarta'</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>SO Devi, AC Irawati</t>
+          <t>AS Sanggacita, H Irhamdessetya, AC Irawati</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Al-Zayn: Jurnal Ilmu Sosial &amp; Hukum 4 (1), 5574-5580, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 283-290, 2026</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -1050,22 +1050,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Penegakan Hukum Tindakan Kriminal Yang Dilakukan Dalam Perjudian Online Oleh Anak-Anak (Studi Kasus Di Kepolisian Metropolitan Semarang)</t>
+          <t>Penerapan Demokrasi Partisipatif Untuk Memperkuat Tata Kelola Desa Yang Baik</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Penegakan Hukum Tindakan Kriminal Yang Dilakukan Dalam Perjudian Online Oleh Anak-Anak (Studi Kasus Di Kepolisian Metropolitan Semarang)'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Penerapan Demokrasi Partisipatif Untuk Memperkuat Tata Kelola Desa Yang Baik'</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AC Irawati</t>
+          <t>KA Saputra, M Lativ, AC Irawati</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 181-190, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 227-233, 2026</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -1081,22 +1081,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Criminal Responsibility of Business Actors for The Distribution of Food Containing Dangerous Substances</t>
+          <t>Keadilan Restoratif: Model Perlindungan Hukum Oleh Aparat Penegak Hukum (Polisi) Dalam Menangani Anak-Anak Yang Terlibat Dalam Perundungan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Criminal Responsibility of Business Actors for The Distribution of Food Containing Dangerous Substances'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Keadilan Restoratif: Model Perlindungan Hukum Oleh Aparat Penegak Hukum (Polisi) Dalam Menangani Anak-Anak Yang Terlibat Dalam Perundungan'</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>W Waryadi, AC Irawati</t>
+          <t>W Winarti, AC Irawati</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>UNTAG Law Review 9 (2), 82-92, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 105-114, 2026</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -1112,22 +1112,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Peran Ahli Patologi Klinis Dalam Memerangi Perdagangan Ilegal Obat Resep Terbatas Di Kabupaten Sleman, Daerah Istimewa Yogyakarta</t>
+          <t>Penegakan Hukum Tindak Pidana Perjudian Melalui Transaksi Informasi dan Elektronik: Studi Putusan Nomor 7104/K/Pid. Sus/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Peran Ahli Patologi Klinis Dalam Memerangi Perdagangan Ilegal Obat Resep Terbatas Di Kabupaten Sleman, Daerah Istimewa Yogyakarta'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Penegakan Hukum Tindak Pidana Perjudian Melalui Transaksi Informasi dan Elektronik: Studi Putusan Nomor 7104/K/Pid. Sus/2025'</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>AS Sanggacita, H Irhamdessetya, AC Irawati</t>
+          <t>SO Devi, AC Irawati</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 283-290, 2026</t>
+          <t>Al-Zayn: Jurnal Ilmu Sosial &amp; Hukum 4 (1), 5574-5580, 2026</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1143,22 +1143,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Penerapan Demokrasi Partisipatif Untuk Memperkuat Tata Kelola Desa Yang Baik</t>
+          <t>Penegakan Hukum Tindakan Kriminal Yang Dilakukan Dalam Perjudian Online Oleh Anak-Anak (Studi Kasus Di Kepolisian Metropolitan Semarang)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Penerapan Demokrasi Partisipatif Untuk Memperkuat Tata Kelola Desa Yang Baik'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Penegakan Hukum Tindakan Kriminal Yang Dilakukan Dalam Perjudian Online Oleh Anak-Anak (Studi Kasus Di Kepolisian Metropolitan Semarang)'</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KA Saputra, M Lativ, AC Irawati</t>
+          <t>AC Irawati</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 227-233, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 181-190, 2026</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -1174,22 +1174,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Keadilan Restoratif: Model Perlindungan Hukum Oleh Aparat Penegak Hukum (Polisi) Dalam Menangani Anak-Anak Yang Terlibat Dalam Perundungan</t>
+          <t>Criminal Responsibility of Business Actors for The Distribution of Food Containing Dangerous Substances</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Keadilan Restoratif: Model Perlindungan Hukum Oleh Aparat Penegak Hukum (Polisi) Dalam Menangani Anak-Anak Yang Terlibat Dalam Perundungan'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Criminal Responsibility of Business Actors for The Distribution of Food Containing Dangerous Substances'</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>W Winarti, AC Irawati</t>
+          <t>W Waryadi, AC Irawati</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 105-114, 2026</t>
+          <t>UNTAG Law Review 9 (2), 82-92, 2026</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -1205,22 +1205,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Model Penegakan Hukum Pada Tindak Pidana Pencurian Anak Melalui Diversi: Studi Putusan Nomor 7/Pid. Sus-Anak/2025/PN Unr</t>
+          <t>Implementasi Ketentuan Batas Usia Dewasa dalam Pelayanan Hukum dan Administrasi Kependudukan pada Pemerintah Desa Mejagong, Kecamatan Randudongkal, Kabupaten Pemalang.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Model Penegakan Hukum Pada Tindak Pidana Pencurian Anak Melalui Diversi: Studi Putusan Nomor 7/Pid. Sus-Anak/2025/PN Unr'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Implementasi Ketentuan Batas Usia Dewasa dalam Pelayanan Hukum dan Administrasi Kependudukan pada Pemerintah Desa Mejagong, Kecamatan Randudongkal, Kabupaten Pemalang.'</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SO Devi, AC Irawati</t>
+          <t>S Sonhaji, AC Irawati</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Al-Zayn: Jurnal Ilmu Sosial &amp; Hukum 4 (1), 5566-5573, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 242-250, 2026</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -1236,29 +1236,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Model Pencegahan Penarikan Kendaraan Leasing Melalui Komunikasi Proaktif Di Kota Semarang</t>
+          <t>Urgensi Kesadaran Digital dalam Mewujudkan Ruang Aman melalui Literasi Digital dan Penerapan Proporsional Undang-Undang ITE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Model Pencegahan Penarikan Kendaraan Leasing Melalui Komunikasi Proaktif Di Kota Semarang'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Urgensi Kesadaran Digital dalam Mewujudkan Ruang Aman melalui Literasi Digital dan Penerapan Proporsional Undang-Undang ITE'</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>RD Saputra, H Irhamdesstya, AC Irawati</t>
+          <t>F Budiarti, H Irhamdesetya, AC Irawati</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 216-226, 2026</t>
+          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 142-151, 2026</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>2026</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1267,22 +1267,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Implementasi E-Faktur Pajak Kendaraan Bermotor dalam Perspektif Hukum Administrasi Negara pada Polrestabes Semarang</t>
+          <t>Penjatuhan Pidana Dalam Tindak Pidana Kekerasan Dalam Rumah Tangga Mewujudkan Kepastian Hukum: Studi Putusan Nomor 121/Pid. Sus/2025/PN Pti</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Implementasi E-Faktur Pajak Kendaraan Bermotor dalam Perspektif Hukum Administrasi Negara pada Polrestabes Semarang'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Penjatuhan Pidana Dalam Tindak Pidana Kekerasan Dalam Rumah Tangga Mewujudkan Kepastian Hukum: Studi Putusan Nomor 121/Pid. Sus/2025/PN Pti'</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>A Wijayanto, AC Irawati</t>
+          <t>QM Ulfa, AC Irawati</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 68-76, 2026</t>
+          <t>Al-Zayn: Jurnal Ilmu Sosial &amp; Hukum 4 (1), 5827-5832, 2026</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -1298,22 +1298,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Implementasi Ketentuan Batas Usia Dewasa dalam Pelayanan Hukum dan Administrasi Kependudukan pada Pemerintah Desa Mejagong, Kecamatan Randudongkal, Kabupaten Pemalang.</t>
+          <t>Model Penegakan Hukum Pada Tindak Pidana Pencurian Anak Melalui Diversi: Studi Putusan Nomor 7/Pid. Sus-Anak/2025/PN Unr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar?q=+intitle:'Implementasi Ketentuan Batas Usia Dewasa dalam Pelayanan Hukum dan Administrasi Kependudukan pada Pemerintah Desa Mejagong, Kecamatan Randudongkal, Kabupaten Pemalang.'</t>
+          <t>https://scholar.google.com/scholar?q=+intitle:'Model Penegakan Hukum Pada Tindak Pidana Pencurian Anak Melalui Diversi: Studi Putusan Nomor 7/Pid. Sus-Anak/2025/PN Unr'</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>S Sonhaji, AC Irawati</t>
+          <t>SO Devi, AC Irawati</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Iuris Studia: Jurnal Kajian Hukum 7 (1), 242-250, 2026</t>
+          <t>Al-Zayn: Jurnal Ilmu Sosial &amp; Hukum 4 (1), 5566-5573, 2026</t>
         </is>
       </c>
       <c r="F11" t="n">

</xml_diff>